<commit_message>
Implementing Individual Salary ChartsVs actual Spent
</commit_message>
<xml_diff>
--- a/temp.xlsx
+++ b/temp.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,11 +518,6 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -573,7 +568,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mother</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -588,7 +583,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Veni Anni Sangam</t>
+          <t>Woman Self Help Group</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -604,18 +599,13 @@
       <c r="Q2" t="inlineStr">
         <is>
           <t>Family</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Note3</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -638,30 +628,30 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Kotak Due</t>
+          <t>Housing Loan</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>4313</v>
+        <v>25633</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>UPI</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Kotak811</t>
+          <t>Gpay</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Chandru</t>
+          <t>Karthi</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -676,7 +666,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Vendor1</t>
+          <t>Bank</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -692,18 +682,13 @@
       <c r="Q3" t="inlineStr">
         <is>
           <t>Family</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>PAID</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-04</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -716,75 +701,1896 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Bike Repair</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Appa</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Yearly</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Local Store</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Skill Development</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Agile Scrum Master Certificate</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>23500</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Imobile</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Chandru</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Chandru</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>One-time</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Anni Recharge</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>199</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Amazon Pay</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Chandru</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Pothu</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Jio</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Loans</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>EMI</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Kotak Due</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>4313</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Bank Transfer</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Kotak811</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Chandru</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Karthi</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Loan</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Anna Recharge</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>349</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Amazon Pay</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Chandru</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Karthi</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Jio</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Home coming</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1050</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Imobile</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Chandru</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Pothu</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Bus Corporation</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Appa Room Rent</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Navi</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Appa</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Appa</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>House Owners</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Loans</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>EMI</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>Kalanchiam Kmpty</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="G11" t="n">
         <v>7000</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Chandru</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Family</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Loan</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Vendor2</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Woman Self Help Group</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Family</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Note2</t>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Medicines</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Physiotherapy</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>500</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Amma</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Medical</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Medical</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>500</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Local Store</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Pongal Things</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>One-time</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Loans</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>EMI</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Azhagu sundari chit fund</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>6400</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Chandru</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Repayment</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Tea &amp;Snacks</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>200</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Navi</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Chandru</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Appa</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Discretionary</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>One-time</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Local Store</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Home coming</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1133</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Imobile</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Karthi</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Karthi</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Bus Corporation</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Poo Veni</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>510</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Amma</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Woman Self Help Group</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Coconut - 10 x 20</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>200</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Local Store</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Hair Oil</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>350</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Amazon Pay</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Discretionary</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>One-time</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Mocha Payir</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>200</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Amma</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Clothes</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Yearly</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Local Store</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Debt</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Interest</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Vairavan</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Deiva</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Repayment</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Fuel</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Appa Bike</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>300</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Kotak811</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Appa</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Medicines</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Patti Tablet</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>150</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Kotak811</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Patti</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Medical</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Act Wifi -BLR</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>883.8200000000001</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Imobile</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Karthi</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Karthi</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Discretionary</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Karthi-House</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>8500</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Karthi</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Karthi</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>House Owners</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Personal</t>
         </is>
       </c>
     </row>
@@ -915,7 +2721,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Karthi</t>
+          <t>Karthi,Deiva</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1006,7 +2812,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GPay</t>
+          <t>Gpay</t>
         </is>
       </c>
     </row>

</xml_diff>